<commit_message>
renew dataset PubOpenShare and update the queryTianyan dataset for institution unmatched
</commit_message>
<xml_diff>
--- a/data-raw/data-tidy/hack-tianyan/hub/match-tianyan-tot-2026-08-hand.xlsx
+++ b/data-raw/data-tidy/hack-tianyan/hub/match-tianyan-tot-2026-08-hand.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\techme\data-raw\data-tidy\hack-tianyan\hub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147D27B3-512C-43DF-9126-658B96FB9522}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F57942B8-30C1-4B21-A06E-785FAE3CFF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11595" yWindow="10740" windowWidth="24420" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="48">
   <si>
     <t>index</t>
   </si>
@@ -284,13 +284,76 @@
   <si>
     <t>金华</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>民政职业大学</t>
+  </si>
+  <si>
+    <t>中国质量检验检测科学研究院</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>北京经济技术开发区荣华南路</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF333333"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>号院</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.tianyancha.com/company/3097987743</t>
+  </si>
+  <si>
+    <t>https://www.tianyancha.com/company/3226931881</t>
+  </si>
+  <si>
+    <r>
+      <t>北京市朝阳区白家庄路甲</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>号</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -397,6 +460,13 @@
       <color rgb="FF333333"/>
       <name val="微软雅黑"/>
       <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333333"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -434,7 +504,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -786,7 +856,7 @@
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" t="s">
         <v>22</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -815,7 +885,7 @@
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" t="s">
         <v>25</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -844,7 +914,7 @@
       <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" t="s">
         <v>29</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -873,7 +943,7 @@
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" t="s">
         <v>32</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -944,17 +1014,63 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D8" s="5"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D9" s="8"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D10" s="5"/>

</xml_diff>